<commit_message>
Updated post processing and footprint calculations, including end of life impact
</commit_message>
<xml_diff>
--- a/Article_data/Step 3 results from Prodcom data manipulations.xlsx
+++ b/Article_data/Step 3 results from Prodcom data manipulations.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nicolas\projects\202604-paper-1-supplementary-code\Article_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80881D6C-5C6C-437D-BBD0-A53F4B769057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1D2142-ADF2-42C6-95CD-FF979A6BD5DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="1000" xr2:uid="{EE4678C9-3BCB-4D41-A2DA-6855614353C7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="1000" activeTab="3" xr2:uid="{EE4678C9-3BCB-4D41-A2DA-6855614353C7}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
     <sheet name="Filtered Prodcom data" sheetId="3" r:id="rId2"/>
     <sheet name="Calculations" sheetId="6" r:id="rId3"/>
-    <sheet name="Hotspots" sheetId="7" r:id="rId4"/>
+    <sheet name="Hotspot prodcom products" sheetId="7" r:id="rId4"/>
     <sheet name="References" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
@@ -9302,9 +9302,6 @@
     <t>Note:</t>
   </si>
   <si>
-    <t>When determining the Ecoinvent regions, if local availability of a product in Europe was 80% or more, we assumed 100% RER or RER w/o RU. See "Get product importers from BACI.ipynb" file in the SI for details on the calculation of import shares from the different regions and countries.</t>
-  </si>
-  <si>
     <t>Prodcom data obtained from "Extract Prodcom data.ipynb"</t>
   </si>
   <si>
@@ -9324,6 +9321,9 @@
   </si>
   <si>
     <t>Ecoinvent 3.12 activity region 5 share</t>
+  </si>
+  <si>
+    <t>When determining the Ecoinvent regions, if local availability of a product in Europe was 80% or more, we assumed 100% RER or RER w/o RU. See "Get product importers from BACI.ipynb" file in the SI for details on the calculation of import shares from the different regions and countries. The table should be exported as CSV and imported into the "Calculate product footprints and generate hotspot figure.ipynb" notebook.</t>
   </si>
 </sst>
 </file>
@@ -9680,7 +9680,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="8" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="9" applyBorder="1" applyAlignment="1">
@@ -9852,9 +9852,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="8" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="13" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -9865,6 +9862,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="15">
@@ -10587,37 +10590,37 @@
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B30" s="86" t="s">
-        <v>3067</v>
-      </c>
-      <c r="C30" s="87" t="str">
+      <c r="B30" s="85" t="s">
+        <v>3066</v>
+      </c>
+      <c r="C30" s="86" t="str">
         <f>'Filtered Prodcom data'!$B$1</f>
         <v>Prodcom data obtained from "Extract Prodcom data.ipynb"</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B31" s="86" t="s">
+      <c r="B31" s="85" t="s">
         <v>2729</v>
       </c>
-      <c r="C31" s="87" t="str">
+      <c r="C31" s="86" t="str">
         <f>Calculations!$B$1</f>
         <v>Data and necessary calculation to split polyamides and isocyanates. Prodcom products into separate product matching with Ecoinvent datasets</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B32" s="86" t="s">
+      <c r="B32" s="85" t="s">
         <v>2730</v>
       </c>
-      <c r="C32" s="87" t="str">
-        <f>Hotspots!$B$1</f>
+      <c r="C32" s="86" t="str">
+        <f>'Hotspot prodcom products'!$B$1</f>
         <v>The table below is an extraction of the table from the previous sheet, taking the top products in the list after screening and ecoinvent matching. Also polyamides and isocyanates were disaggregated below</v>
       </c>
     </row>
     <row r="33" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="88" t="s">
+      <c r="B33" s="87" t="s">
         <v>2731</v>
       </c>
-      <c r="C33" s="89" t="str">
+      <c r="C33" s="88" t="str">
         <f>References!$B$1</f>
         <v>Bibliography: list of references used thoughout the workbook</v>
       </c>
@@ -10893,7 +10896,7 @@
         <v>3061</v>
       </c>
       <c r="B1" s="50" t="s">
-        <v>3065</v>
+        <v>3064</v>
       </c>
       <c r="AC1" s="44"/>
       <c r="AE1" s="44"/>
@@ -10906,7 +10909,7 @@
         <v>3063</v>
       </c>
       <c r="B2" s="50" t="s">
-        <v>3066</v>
+        <v>3065</v>
       </c>
       <c r="AC2" s="44"/>
       <c r="AE2" s="44"/>
@@ -39911,7 +39914,7 @@
         <v>3061</v>
       </c>
       <c r="B1" t="s">
-        <v>3068</v>
+        <v>3067</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="50" customFormat="1" x14ac:dyDescent="0.3"/>
@@ -40255,16 +40258,16 @@
       <c r="A2" t="s">
         <v>3063</v>
       </c>
-      <c r="B2" t="s">
-        <v>3064</v>
+      <c r="B2" s="91" t="s">
+        <v>3071</v>
       </c>
     </row>
     <row r="3" spans="1:31" s="50" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="F4" s="85" t="s">
+      <c r="F4" s="90" t="s">
         <v>705</v>
       </c>
-      <c r="G4" s="85"/>
+      <c r="G4" s="90"/>
       <c r="I4" s="47"/>
       <c r="J4" s="47"/>
     </row>
@@ -40357,10 +40360,10 @@
         <v>3056</v>
       </c>
       <c r="AD5" s="57" t="s">
+        <v>3069</v>
+      </c>
+      <c r="AE5" s="57" t="s">
         <v>3070</v>
-      </c>
-      <c r="AE5" s="57" t="s">
-        <v>3071</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.3">
@@ -40670,8 +40673,8 @@
       <c r="B10" t="s">
         <v>111</v>
       </c>
-      <c r="C10" s="90" t="s">
-        <v>3069</v>
+      <c r="C10" s="89" t="s">
+        <v>3068</v>
       </c>
       <c r="D10" t="s">
         <v>112</v>

</xml_diff>

<commit_message>
Update step 3 excel
</commit_message>
<xml_diff>
--- a/Article_data/Step 3 results from Prodcom data manipulations.xlsx
+++ b/Article_data/Step 3 results from Prodcom data manipulations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nicolas\projects\202604-paper-1-supplementary-code\Article_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA3D65E2-710E-4C0C-B3E1-BDBBEB851D94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D6E6228-23B6-4D98-B031-21ED139D87E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="570" activeTab="2" xr2:uid="{EE4678C9-3BCB-4D41-A2DA-6855614353C7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="570" xr2:uid="{EE4678C9-3BCB-4D41-A2DA-6855614353C7}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -8756,9 +8756,6 @@
     <t>(Prohaska et al., 2022, p. 581)</t>
   </si>
   <si>
-    <t>The table below is an extraction of the table from the previous sheet, taking the top products in the list after screening and ecoinvent matching. Also polyamides and isocyanates were disaggregated below</t>
-  </si>
-  <si>
     <t>PRODCOM code</t>
   </si>
   <si>
@@ -9336,6 +9333,9 @@
   </si>
   <si>
     <t>Hotspot products export</t>
+  </si>
+  <si>
+    <t>The table below is an extraction of the table from the previous sheet, taking the top products in the list after screening and ecoinvent matching. Also polyamides and isocyanates were disaggregated below. Table to be exported for use as input CSV in the footprint calculation notebook.</t>
   </si>
 </sst>
 </file>
@@ -10585,7 +10585,7 @@
         <v>46245</v>
       </c>
       <c r="C23" s="29" t="s">
-        <v>3058</v>
+        <v>3057</v>
       </c>
     </row>
     <row r="24" spans="2:3" s="50" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -10593,7 +10593,7 @@
         <v>46247</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>3074</v>
+        <v>3073</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="18" thickBot="1" x14ac:dyDescent="0.4">
@@ -10620,7 +10620,7 @@
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B31" s="85" t="s">
-        <v>3064</v>
+        <v>3063</v>
       </c>
       <c r="C31" s="86" t="str">
         <f>'Filtered Prodcom data'!$B$1</f>
@@ -10638,11 +10638,11 @@
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B33" s="85" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
       <c r="C33" s="86" t="str">
         <f>'Hotspot products export'!$B$1</f>
-        <v>The table below is an extraction of the table from the previous sheet, taking the top products in the list after screening and ecoinvent matching. Also polyamides and isocyanates were disaggregated below</v>
+        <v>The table below is an extraction of the table from the previous sheet, taking the top products in the list after screening and ecoinvent matching. Also polyamides and isocyanates were disaggregated below. Table to be exported for use as input CSV in the footprint calculation notebook.</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -10922,10 +10922,10 @@
   <sheetData>
     <row r="1" spans="1:37" s="50" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="50" t="s">
-        <v>3059</v>
+        <v>3058</v>
       </c>
       <c r="B1" s="50" t="s">
-        <v>3062</v>
+        <v>3061</v>
       </c>
       <c r="AC1" s="44"/>
       <c r="AE1" s="44"/>
@@ -10935,10 +10935,10 @@
     </row>
     <row r="2" spans="1:37" s="50" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="50" t="s">
-        <v>3061</v>
+        <v>3060</v>
       </c>
       <c r="B2" s="50" t="s">
-        <v>3063</v>
+        <v>3062</v>
       </c>
       <c r="AC2" s="44"/>
       <c r="AE2" s="44"/>
@@ -39940,10 +39940,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="50" t="s">
-        <v>3059</v>
+        <v>3058</v>
       </c>
       <c r="B1" t="s">
-        <v>3065</v>
+        <v>3064</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="50" customFormat="1" x14ac:dyDescent="0.3"/>
@@ -39968,7 +39968,7 @@
         <v>2370412440</v>
       </c>
       <c r="D6" s="53" t="s">
-        <v>3032</v>
+        <v>3031</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -40192,7 +40192,7 @@
         <v>1049281862</v>
       </c>
       <c r="D32" s="53" t="s">
-        <v>3032</v>
+        <v>3031</v>
       </c>
     </row>
     <row r="34" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.4">
@@ -40277,26 +40277,26 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="50" t="s">
-        <v>3059</v>
+        <v>3058</v>
       </c>
       <c r="B1" t="s">
-        <v>2882</v>
+        <v>3075</v>
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>3061</v>
+        <v>3060</v>
       </c>
       <c r="B2" s="90" t="s">
-        <v>3069</v>
+        <v>3068</v>
       </c>
     </row>
     <row r="3" spans="1:31" s="50" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="50" t="s">
+        <v>3071</v>
+      </c>
+      <c r="B3" s="50" t="s">
         <v>3072</v>
-      </c>
-      <c r="B3" s="50" t="s">
-        <v>3073</v>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.3">
@@ -40305,103 +40305,103 @@
       </c>
       <c r="G4" s="92"/>
       <c r="I4" s="47" t="s">
-        <v>3071</v>
+        <v>3070</v>
       </c>
       <c r="J4" s="47"/>
     </row>
     <row r="5" spans="1:31" s="15" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A5" s="91" t="s">
-        <v>3056</v>
+        <v>3055</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>2883</v>
+        <v>2882</v>
       </c>
       <c r="C5" s="57" t="s">
         <v>2808</v>
       </c>
       <c r="D5" s="57" t="s">
+        <v>2883</v>
+      </c>
+      <c r="E5" s="57" t="s">
         <v>2884</v>
       </c>
-      <c r="E5" s="57" t="s">
-        <v>2885</v>
-      </c>
       <c r="F5" s="57" t="s">
+        <v>3032</v>
+      </c>
+      <c r="G5" s="57" t="s">
         <v>3033</v>
       </c>
-      <c r="G5" s="57" t="s">
-        <v>3034</v>
-      </c>
       <c r="H5" s="57" t="s">
-        <v>3057</v>
+        <v>3056</v>
       </c>
       <c r="I5" s="91" t="s">
-        <v>3070</v>
+        <v>3069</v>
       </c>
       <c r="J5" s="57" t="s">
         <v>2617</v>
       </c>
       <c r="K5" s="57" t="s">
+        <v>2885</v>
+      </c>
+      <c r="L5" s="57" t="s">
         <v>2886</v>
       </c>
-      <c r="L5" s="57" t="s">
+      <c r="M5" s="57" t="s">
         <v>2887</v>
       </c>
-      <c r="M5" s="57" t="s">
+      <c r="N5" s="57" t="s">
         <v>2888</v>
       </c>
-      <c r="N5" s="57" t="s">
+      <c r="O5" s="62" t="s">
         <v>2889</v>
       </c>
-      <c r="O5" s="62" t="s">
-        <v>2890</v>
-      </c>
       <c r="P5" s="57" t="s">
+        <v>3034</v>
+      </c>
+      <c r="Q5" s="57" t="s">
         <v>3035</v>
       </c>
-      <c r="Q5" s="57" t="s">
-        <v>3036</v>
-      </c>
       <c r="R5" s="57" t="s">
+        <v>3037</v>
+      </c>
+      <c r="S5" s="57" t="s">
         <v>3038</v>
       </c>
-      <c r="S5" s="57" t="s">
+      <c r="T5" s="57" t="s">
+        <v>3047</v>
+      </c>
+      <c r="U5" s="62" t="s">
+        <v>3048</v>
+      </c>
+      <c r="V5" s="57" t="s">
+        <v>3040</v>
+      </c>
+      <c r="W5" s="57" t="s">
+        <v>3041</v>
+      </c>
+      <c r="X5" s="57" t="s">
         <v>3039</v>
       </c>
-      <c r="T5" s="57" t="s">
-        <v>3048</v>
-      </c>
-      <c r="U5" s="62" t="s">
+      <c r="Y5" s="57" t="s">
+        <v>3045</v>
+      </c>
+      <c r="Z5" s="57" t="s">
         <v>3049</v>
       </c>
-      <c r="V5" s="57" t="s">
-        <v>3041</v>
-      </c>
-      <c r="W5" s="57" t="s">
-        <v>3042</v>
-      </c>
-      <c r="X5" s="57" t="s">
-        <v>3040</v>
-      </c>
-      <c r="Y5" s="57" t="s">
-        <v>3046</v>
-      </c>
-      <c r="Z5" s="57" t="s">
+      <c r="AA5" s="57" t="s">
         <v>3050</v>
       </c>
-      <c r="AA5" s="57" t="s">
-        <v>3051</v>
-      </c>
       <c r="AB5" s="57" t="s">
+        <v>3052</v>
+      </c>
+      <c r="AC5" s="57" t="s">
         <v>3053</v>
       </c>
-      <c r="AC5" s="57" t="s">
-        <v>3054</v>
-      </c>
       <c r="AD5" s="57" t="s">
+        <v>3066</v>
+      </c>
+      <c r="AE5" s="57" t="s">
         <v>3067</v>
-      </c>
-      <c r="AE5" s="57" t="s">
-        <v>3068</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.3">
@@ -40418,7 +40418,7 @@
         <v>615</v>
       </c>
       <c r="E6" s="48" t="s">
-        <v>2891</v>
+        <v>2890</v>
       </c>
       <c r="F6" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B6, prodcom_data[product], 0))</f>
@@ -40439,23 +40439,23 @@
         <v>2642</v>
       </c>
       <c r="K6" s="79" t="s">
-        <v>2892</v>
+        <v>2891</v>
       </c>
       <c r="L6" s="79">
         <v>42.081000000000003</v>
       </c>
       <c r="M6" s="80" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="N6" s="72">
         <f>M6*Calculations!$C$37/L6</f>
         <v>0.85627717972481643</v>
       </c>
       <c r="O6" s="81" t="s">
-        <v>2894</v>
+        <v>2893</v>
       </c>
       <c r="P6" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q6" s="58">
         <v>1</v>
@@ -40465,7 +40465,7 @@
       <c r="T6" s="59"/>
       <c r="U6" s="63"/>
       <c r="V6" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W6" s="58">
         <v>1</v>
@@ -40514,23 +40514,23 @@
         <v>2642</v>
       </c>
       <c r="K7" s="79" t="s">
-        <v>2898</v>
+        <v>2897</v>
       </c>
       <c r="L7" s="79">
         <v>28.05</v>
       </c>
       <c r="M7" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N7" s="72">
         <f>M7*Calculations!$C$37/L7</f>
         <v>0.85639928698752221</v>
       </c>
       <c r="O7" s="81" t="s">
-        <v>2900</v>
+        <v>2899</v>
       </c>
       <c r="P7" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q7" s="58">
         <v>1</v>
@@ -40540,7 +40540,7 @@
       <c r="T7" s="59"/>
       <c r="U7" s="63"/>
       <c r="V7" s="59" t="s">
-        <v>3045</v>
+        <v>3044</v>
       </c>
       <c r="W7" s="58">
         <v>1</v>
@@ -40568,7 +40568,7 @@
         <v>12</v>
       </c>
       <c r="E8" s="48" t="s">
-        <v>2895</v>
+        <v>2894</v>
       </c>
       <c r="F8" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B8, prodcom_data[product], 0))</f>
@@ -40589,23 +40589,23 @@
         <v>2642</v>
       </c>
       <c r="K8" s="79" t="s">
-        <v>2896</v>
+        <v>2895</v>
       </c>
       <c r="L8" s="79">
         <v>42.08</v>
       </c>
       <c r="M8" s="80" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="N8" s="72">
         <f>M8*Calculations!$C$37/L8</f>
         <v>0.85629752851711038</v>
       </c>
       <c r="O8" s="81" t="s">
-        <v>2897</v>
+        <v>2896</v>
       </c>
       <c r="P8" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q8" s="58">
         <v>1</v>
@@ -40615,7 +40615,7 @@
       <c r="T8" s="59"/>
       <c r="U8" s="63"/>
       <c r="V8" s="59" t="s">
-        <v>3045</v>
+        <v>3044</v>
       </c>
       <c r="W8" s="58">
         <v>1</v>
@@ -40643,7 +40643,7 @@
         <v>540</v>
       </c>
       <c r="E9" s="48" t="s">
-        <v>2901</v>
+        <v>2900</v>
       </c>
       <c r="F9" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B9, prodcom_data[product], 0))</f>
@@ -40664,23 +40664,23 @@
         <v>2642</v>
       </c>
       <c r="K9" s="79" t="s">
-        <v>2902</v>
+        <v>2901</v>
       </c>
       <c r="L9" s="79">
         <v>28.053999999999998</v>
       </c>
       <c r="M9" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N9" s="72">
         <f>M9*Calculations!$C$37/L9</f>
         <v>0.85627717972481643</v>
       </c>
       <c r="O9" s="81" t="s">
-        <v>2903</v>
+        <v>2902</v>
       </c>
       <c r="P9" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q9" s="58">
         <v>1</v>
@@ -40690,7 +40690,7 @@
       <c r="T9" s="59"/>
       <c r="U9" s="63"/>
       <c r="V9" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W9" s="58">
         <v>1</v>
@@ -40712,13 +40712,13 @@
         <v>111</v>
       </c>
       <c r="C10" s="89" t="s">
-        <v>3066</v>
+        <v>3065</v>
       </c>
       <c r="D10" t="s">
         <v>112</v>
       </c>
       <c r="E10" s="48" t="s">
-        <v>2904</v>
+        <v>2903</v>
       </c>
       <c r="F10" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B10, prodcom_data[product], 0))</f>
@@ -40739,66 +40739,66 @@
         <v>2642</v>
       </c>
       <c r="K10" s="79" t="s">
-        <v>2905</v>
+        <v>2904</v>
       </c>
       <c r="L10" s="79">
         <v>32.042000000000002</v>
       </c>
       <c r="M10" s="80" t="s">
-        <v>2906</v>
+        <v>2905</v>
       </c>
       <c r="N10" s="72">
         <f>M10*Calculations!$C$37/L10</f>
         <v>0.3748517570688471</v>
       </c>
       <c r="O10" s="81" t="s">
-        <v>2907</v>
+        <v>2906</v>
       </c>
       <c r="P10" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q10" s="58">
         <v>0.35</v>
       </c>
       <c r="R10" s="59" t="s">
-        <v>3047</v>
+        <v>3046</v>
       </c>
       <c r="S10" s="58">
         <v>0.23</v>
       </c>
       <c r="T10" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="U10" s="61">
         <f>1-Q10-S10</f>
         <v>0.42000000000000004</v>
       </c>
       <c r="V10" s="59" t="s">
-        <v>3045</v>
+        <v>3044</v>
       </c>
       <c r="W10" s="58">
         <v>0.18</v>
       </c>
       <c r="X10" s="59" t="s">
-        <v>3052</v>
+        <v>3051</v>
       </c>
       <c r="Y10" s="58">
         <v>0.21</v>
       </c>
       <c r="Z10" s="59" t="s">
-        <v>3047</v>
+        <v>3046</v>
       </c>
       <c r="AA10" s="58">
         <v>0.23</v>
       </c>
       <c r="AB10" s="59" t="s">
-        <v>3055</v>
+        <v>3054</v>
       </c>
       <c r="AC10" s="60">
         <v>0.16</v>
       </c>
       <c r="AD10" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="AE10" s="61" cm="1">
         <f t="array" ref="AE10">1-SUM(IF(ISNUMBER(V10:AC10), V10:AC10, 0))</f>
@@ -40840,23 +40840,23 @@
         <v>2642</v>
       </c>
       <c r="K11" s="79" t="s">
-        <v>2908</v>
+        <v>2907</v>
       </c>
       <c r="L11" s="79">
         <v>78.11</v>
       </c>
       <c r="M11" s="80" t="s">
-        <v>2909</v>
+        <v>2908</v>
       </c>
       <c r="N11" s="72">
         <f>M11*Calculations!$C$37/L11</f>
         <v>0.92262194341313541</v>
       </c>
       <c r="O11" s="81" t="s">
-        <v>2910</v>
+        <v>2909</v>
       </c>
       <c r="P11" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q11" s="58">
         <v>1</v>
@@ -40866,7 +40866,7 @@
       <c r="T11" s="59"/>
       <c r="U11" s="63"/>
       <c r="V11" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W11" s="58">
         <v>1</v>
@@ -40894,7 +40894,7 @@
         <v>564</v>
       </c>
       <c r="E12" s="48" t="s">
-        <v>2911</v>
+        <v>2910</v>
       </c>
       <c r="F12" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B12, prodcom_data[product], 0))</f>
@@ -40915,23 +40915,23 @@
         <v>2642</v>
       </c>
       <c r="K12" s="79" t="s">
-        <v>2912</v>
+        <v>2911</v>
       </c>
       <c r="L12" s="79">
         <v>62.5</v>
       </c>
       <c r="M12" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N12" s="72">
         <f>M12*Calculations!$C$37/L12</f>
         <v>0.38435199999999997</v>
       </c>
       <c r="O12" s="81" t="s">
-        <v>2913</v>
+        <v>2912</v>
       </c>
       <c r="P12" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q12" s="58">
         <v>1</v>
@@ -40941,7 +40941,7 @@
       <c r="T12" s="59"/>
       <c r="U12" s="63"/>
       <c r="V12" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W12" s="58">
         <v>1</v>
@@ -40969,7 +40969,7 @@
         <v>537</v>
       </c>
       <c r="E13" s="48" t="s">
-        <v>2901</v>
+        <v>2900</v>
       </c>
       <c r="F13" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B13, prodcom_data[product], 0))</f>
@@ -40990,23 +40990,23 @@
         <v>2642</v>
       </c>
       <c r="K13" s="79" t="s">
-        <v>2902</v>
+        <v>2901</v>
       </c>
       <c r="L13" s="79">
         <v>28.053999999999998</v>
       </c>
       <c r="M13" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N13" s="72">
         <f>M13*Calculations!$C$37/L13</f>
         <v>0.85627717972481643</v>
       </c>
       <c r="O13" s="81" t="s">
-        <v>2903</v>
+        <v>2902</v>
       </c>
       <c r="P13" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q13" s="58">
         <v>1</v>
@@ -41016,7 +41016,7 @@
       <c r="T13" s="59"/>
       <c r="U13" s="63"/>
       <c r="V13" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W13" s="58">
         <v>1</v>
@@ -41044,7 +41044,7 @@
         <v>534</v>
       </c>
       <c r="E14" s="48" t="s">
-        <v>2901</v>
+        <v>2900</v>
       </c>
       <c r="F14" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B14, prodcom_data[product], 0))</f>
@@ -41065,23 +41065,23 @@
         <v>2642</v>
       </c>
       <c r="K14" s="79" t="s">
-        <v>2902</v>
+        <v>2901</v>
       </c>
       <c r="L14" s="79">
         <v>28.053999999999998</v>
       </c>
       <c r="M14" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N14" s="72">
         <f>M14*Calculations!$C$37/L14</f>
         <v>0.85627717972481643</v>
       </c>
       <c r="O14" s="81" t="s">
-        <v>2903</v>
+        <v>2902</v>
       </c>
       <c r="P14" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q14" s="58">
         <v>1</v>
@@ -41091,7 +41091,7 @@
       <c r="T14" s="59"/>
       <c r="U14" s="63"/>
       <c r="V14" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W14" s="58">
         <v>1</v>
@@ -41140,23 +41140,23 @@
         <v>2642</v>
       </c>
       <c r="K15" s="79" t="s">
-        <v>2922</v>
+        <v>2921</v>
       </c>
       <c r="L15" s="79">
         <v>104.15</v>
       </c>
       <c r="M15" s="80" t="s">
-        <v>2916</v>
+        <v>2915</v>
       </c>
       <c r="N15" s="72">
         <f>M15*Calculations!$C$37/L15</f>
         <v>0.92259241478636567</v>
       </c>
       <c r="O15" s="81" t="s">
-        <v>2923</v>
+        <v>2922</v>
       </c>
       <c r="P15" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q15" s="58">
         <v>1</v>
@@ -41166,7 +41166,7 @@
       <c r="T15" s="59"/>
       <c r="U15" s="63"/>
       <c r="V15" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W15" s="58">
         <v>1</v>
@@ -41194,7 +41194,7 @@
         <v>264</v>
       </c>
       <c r="E16" s="48" t="s">
-        <v>2914</v>
+        <v>2913</v>
       </c>
       <c r="F16" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B16, prodcom_data[product], 0))</f>
@@ -41215,23 +41215,23 @@
         <v>2656</v>
       </c>
       <c r="K16" s="79" t="s">
-        <v>2915</v>
+        <v>2914</v>
       </c>
       <c r="L16" s="79">
         <v>166.13</v>
       </c>
       <c r="M16" s="80" t="s">
-        <v>2916</v>
+        <v>2915</v>
       </c>
       <c r="N16" s="72">
         <f>M16*Calculations!$C$37/L16</f>
         <v>0.57839041714320105</v>
       </c>
       <c r="O16" s="81" t="s">
-        <v>2917</v>
+        <v>2916</v>
       </c>
       <c r="P16" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q16" s="58">
         <v>1</v>
@@ -41241,7 +41241,7 @@
       <c r="T16" s="59"/>
       <c r="U16" s="63"/>
       <c r="V16" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W16" s="58">
         <v>1</v>
@@ -41269,7 +41269,7 @@
         <v>600</v>
       </c>
       <c r="E17" s="48" t="s">
-        <v>2918</v>
+        <v>2917</v>
       </c>
       <c r="F17" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B17, prodcom_data[product], 0))</f>
@@ -41290,23 +41290,23 @@
         <v>2642</v>
       </c>
       <c r="K17" s="79" t="s">
-        <v>2919</v>
+        <v>2918</v>
       </c>
       <c r="L17" s="79">
         <v>222.24</v>
       </c>
       <c r="M17" s="80" t="s">
-        <v>2920</v>
+        <v>2919</v>
       </c>
       <c r="N17" s="72">
         <f>M17*Calculations!$C$37/L17</f>
         <v>0.64854211663066952</v>
       </c>
       <c r="O17" s="81" t="s">
-        <v>2921</v>
+        <v>2920</v>
       </c>
       <c r="P17" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q17" s="58">
         <v>1</v>
@@ -41316,7 +41316,7 @@
       <c r="T17" s="59"/>
       <c r="U17" s="63"/>
       <c r="V17" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W17" s="58">
         <v>1</v>
@@ -41344,7 +41344,7 @@
         <v>18</v>
       </c>
       <c r="E18" s="48" t="s">
-        <v>2924</v>
+        <v>2923</v>
       </c>
       <c r="F18" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B18, prodcom_data[product], 0))</f>
@@ -41365,23 +41365,23 @@
         <v>2660</v>
       </c>
       <c r="K18" s="79" t="s">
-        <v>2925</v>
+        <v>2924</v>
       </c>
       <c r="L18" s="79">
         <v>54.09</v>
       </c>
       <c r="M18" s="80" t="s">
-        <v>2926</v>
+        <v>2925</v>
       </c>
       <c r="N18" s="72">
         <f>M18*Calculations!$C$37/L18</f>
         <v>0.88822333148456267</v>
       </c>
       <c r="O18" s="81" t="s">
-        <v>2927</v>
+        <v>2926</v>
       </c>
       <c r="P18" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q18" s="58">
         <v>1</v>
@@ -41391,7 +41391,7 @@
       <c r="T18" s="59"/>
       <c r="U18" s="63"/>
       <c r="V18" s="59" t="s">
-        <v>3045</v>
+        <v>3044</v>
       </c>
       <c r="W18" s="58">
         <v>1</v>
@@ -41419,7 +41419,7 @@
         <v>15</v>
       </c>
       <c r="E19" s="48" t="s">
-        <v>2928</v>
+        <v>2927</v>
       </c>
       <c r="F19" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B19, prodcom_data[product], 0))</f>
@@ -41440,23 +41440,23 @@
         <v>2642</v>
       </c>
       <c r="K19" s="79" t="s">
-        <v>2929</v>
+        <v>2928</v>
       </c>
       <c r="L19" s="79">
         <v>112.21</v>
       </c>
       <c r="M19" s="80" t="s">
-        <v>2916</v>
+        <v>2915</v>
       </c>
       <c r="N19" s="72">
         <f>M19*Calculations!$C$37/L19</f>
         <v>0.85632296586756973</v>
       </c>
       <c r="O19" s="81" t="s">
-        <v>2930</v>
+        <v>2929</v>
       </c>
       <c r="P19" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q19" s="58">
         <v>1</v>
@@ -41466,7 +41466,7 @@
       <c r="T19" s="59"/>
       <c r="U19" s="63"/>
       <c r="V19" s="59" t="s">
-        <v>3045</v>
+        <v>3044</v>
       </c>
       <c r="W19" s="58">
         <v>1</v>
@@ -41494,7 +41494,7 @@
         <v>549</v>
       </c>
       <c r="E20" s="48" t="s">
-        <v>2931</v>
+        <v>2930</v>
       </c>
       <c r="F20" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B20, prodcom_data[product], 0))</f>
@@ -41515,23 +41515,23 @@
         <v>2642</v>
       </c>
       <c r="K20" s="79" t="s">
-        <v>2932</v>
+        <v>2931</v>
       </c>
       <c r="L20" s="79">
         <v>104.15199999999999</v>
       </c>
       <c r="M20" s="80" t="s">
-        <v>2916</v>
+        <v>2915</v>
       </c>
       <c r="N20" s="72">
         <f>M20*Calculations!$C$37/L20</f>
         <v>0.92257469851755136</v>
       </c>
       <c r="O20" s="81" t="s">
-        <v>2933</v>
+        <v>2932</v>
       </c>
       <c r="P20" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q20" s="58">
         <v>1</v>
@@ -41541,7 +41541,7 @@
       <c r="T20" s="59"/>
       <c r="U20" s="63"/>
       <c r="V20" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W20" s="58">
         <v>1</v>
@@ -41569,7 +41569,7 @@
         <v>133</v>
       </c>
       <c r="E21" s="48" t="s">
-        <v>2937</v>
+        <v>2936</v>
       </c>
       <c r="F21" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B21, prodcom_data[product], 0))</f>
@@ -41590,29 +41590,29 @@
         <v>2642</v>
       </c>
       <c r="K21" s="79" t="s">
-        <v>2938</v>
+        <v>2937</v>
       </c>
       <c r="L21" s="79">
         <v>62.07</v>
       </c>
       <c r="M21" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N21" s="72">
         <f>M21*Calculations!$C$37/L21</f>
         <v>0.38701466086676328</v>
       </c>
       <c r="O21" s="81" t="s">
-        <v>2939</v>
+        <v>2938</v>
       </c>
       <c r="P21" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q21" s="60">
         <v>0.56000000000000005</v>
       </c>
       <c r="R21" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S21" s="61" cm="1">
         <f t="array" ref="S21">1-SUM(IF(ISNUMBER(P21:Q21), P21:Q21, 0))</f>
@@ -41621,13 +41621,13 @@
       <c r="T21" s="59"/>
       <c r="U21" s="63"/>
       <c r="V21" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W21" s="60">
         <v>0.56000000000000005</v>
       </c>
       <c r="X21" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y21" s="61" cm="1">
         <f t="array" ref="Y21">1-SUM(IF(ISNUMBER(V21:W21), V21:W21, 0))</f>
@@ -41654,7 +41654,7 @@
         <v>477</v>
       </c>
       <c r="E22" s="48" t="s">
-        <v>2934</v>
+        <v>2933</v>
       </c>
       <c r="F22" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B22, prodcom_data[product], 0))</f>
@@ -41675,23 +41675,23 @@
         <v>2642</v>
       </c>
       <c r="K22" s="79" t="s">
-        <v>2935</v>
+        <v>2934</v>
       </c>
       <c r="L22" s="79">
         <v>58.08</v>
       </c>
       <c r="M22" s="80" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="N22" s="72">
         <f>M22*Calculations!$C$37/L22</f>
         <v>0.62040289256198355</v>
       </c>
       <c r="O22" s="81" t="s">
-        <v>2936</v>
+        <v>2935</v>
       </c>
       <c r="P22" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q22" s="58">
         <v>1</v>
@@ -41701,7 +41701,7 @@
       <c r="T22" s="59"/>
       <c r="U22" s="63"/>
       <c r="V22" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W22" s="58">
         <v>1</v>
@@ -41729,7 +41729,7 @@
         <v>552</v>
       </c>
       <c r="E23" s="48" t="s">
-        <v>2931</v>
+        <v>2930</v>
       </c>
       <c r="F23" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B23, prodcom_data[product], 0))</f>
@@ -41750,23 +41750,23 @@
         <v>2642</v>
       </c>
       <c r="K23" s="79" t="s">
-        <v>2932</v>
+        <v>2931</v>
       </c>
       <c r="L23" s="79">
         <v>104.15199999999999</v>
       </c>
       <c r="M23" s="80" t="s">
-        <v>2916</v>
+        <v>2915</v>
       </c>
       <c r="N23" s="72">
         <f>M23*Calculations!$C$37/L23</f>
         <v>0.92257469851755136</v>
       </c>
       <c r="O23" s="81" t="s">
-        <v>2933</v>
+        <v>2932</v>
       </c>
       <c r="P23" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q23" s="58">
         <v>1</v>
@@ -41776,7 +41776,7 @@
       <c r="T23" s="59"/>
       <c r="U23" s="63"/>
       <c r="V23" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W23" s="58">
         <v>1</v>
@@ -41804,7 +41804,7 @@
         <v>73</v>
       </c>
       <c r="E24" s="48" t="s">
-        <v>2944</v>
+        <v>2943</v>
       </c>
       <c r="F24" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B24, prodcom_data[product], 0))</f>
@@ -41825,29 +41825,29 @@
         <v>2642</v>
       </c>
       <c r="K24" s="79" t="s">
-        <v>2945</v>
+        <v>2944</v>
       </c>
       <c r="L24" s="79">
         <v>98.96</v>
       </c>
       <c r="M24" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N24" s="72">
         <f>M24*Calculations!$C$37/L24</f>
         <v>0.24274454324979791</v>
       </c>
       <c r="O24" s="81" t="s">
-        <v>2946</v>
+        <v>2945</v>
       </c>
       <c r="P24" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q24" s="58">
         <v>0.86</v>
       </c>
       <c r="R24" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S24" s="61" cm="1">
         <f t="array" ref="S24">1-SUM(IF(ISNUMBER(P24:Q24), P24:Q24, 0))</f>
@@ -41856,13 +41856,13 @@
       <c r="T24" s="59"/>
       <c r="U24" s="63"/>
       <c r="V24" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W24" s="58">
         <v>0.86</v>
       </c>
       <c r="X24" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y24" s="61" cm="1">
         <f t="array" ref="Y24">1-SUM(IF(ISNUMBER(V24:W24), V24:W24, 0))</f>
@@ -41910,29 +41910,29 @@
         <v>2642</v>
       </c>
       <c r="K25" s="79" t="s">
-        <v>2981</v>
+        <v>2980</v>
       </c>
       <c r="L25" s="79">
         <v>106.16</v>
       </c>
       <c r="M25" s="80" t="s">
-        <v>2916</v>
+        <v>2915</v>
       </c>
       <c r="N25" s="72">
         <f>M25*Calculations!$C$37/L25</f>
         <v>0.90512434061793512</v>
       </c>
       <c r="O25" s="81" t="s">
-        <v>2982</v>
+        <v>2981</v>
       </c>
       <c r="P25" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q25" s="58">
         <v>0.48</v>
       </c>
       <c r="R25" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S25" s="61" cm="1">
         <f t="array" ref="S25">1-SUM(IF(ISNUMBER(P25:Q25), P25:Q25, 0))</f>
@@ -41941,13 +41941,13 @@
       <c r="T25" s="59"/>
       <c r="U25" s="63"/>
       <c r="V25" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W25" s="58">
         <v>0.48</v>
       </c>
       <c r="X25" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y25" s="61" cm="1">
         <f t="array" ref="Y25">1-SUM(IF(ISNUMBER(V25:W25), V25:W25, 0))</f>
@@ -41995,23 +41995,23 @@
         <v>2642</v>
       </c>
       <c r="K26" s="79" t="s">
-        <v>2947</v>
+        <v>2946</v>
       </c>
       <c r="L26" s="79">
         <v>92.14</v>
       </c>
       <c r="M26" s="80" t="s">
-        <v>2948</v>
+        <v>2947</v>
       </c>
       <c r="N26" s="72">
         <f>M26*Calculations!$C$37/L26</f>
         <v>0.91249186021271977</v>
       </c>
       <c r="O26" s="81" t="s">
-        <v>2949</v>
+        <v>2948</v>
       </c>
       <c r="P26" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q26" s="58">
         <v>1</v>
@@ -42021,7 +42021,7 @@
       <c r="T26" s="59"/>
       <c r="U26" s="63"/>
       <c r="V26" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W26" s="58">
         <v>1</v>
@@ -42070,29 +42070,29 @@
         <v>2642</v>
       </c>
       <c r="K27" s="79" t="s">
-        <v>2935</v>
+        <v>2934</v>
       </c>
       <c r="L27" s="79">
         <v>58.08</v>
       </c>
       <c r="M27" s="80" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="N27" s="72">
         <f>M27*Calculations!$C$37/L27</f>
         <v>0.62040289256198355</v>
       </c>
       <c r="O27" s="81" t="s">
-        <v>2943</v>
+        <v>2942</v>
       </c>
       <c r="P27" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q27" s="58">
         <v>0.93</v>
       </c>
       <c r="R27" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S27" s="61" cm="1">
         <f t="array" ref="S27">1-SUM(IF(ISNUMBER(P27:Q27), P27:Q27, 0))</f>
@@ -42101,13 +42101,13 @@
       <c r="T27" s="59"/>
       <c r="U27" s="63"/>
       <c r="V27" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W27" s="58">
         <v>0.93</v>
       </c>
       <c r="X27" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y27" s="61" cm="1">
         <f t="array" ref="Y27">1-SUM(IF(ISNUMBER(V27:W27), V27:W27, 0))</f>
@@ -42134,7 +42134,7 @@
         <v>388</v>
       </c>
       <c r="E28" s="48" t="s">
-        <v>2953</v>
+        <v>2952</v>
       </c>
       <c r="F28" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B28, prodcom_data[product], 0))</f>
@@ -42155,23 +42155,23 @@
         <v>2642</v>
       </c>
       <c r="K28" s="79" t="s">
-        <v>2954</v>
+        <v>2953</v>
       </c>
       <c r="L28" s="79">
         <v>30.026</v>
       </c>
       <c r="M28" s="80" t="s">
-        <v>2906</v>
+        <v>2905</v>
       </c>
       <c r="N28" s="72">
         <f>M28*Calculations!$C$37/L28</f>
         <v>0.40001998268167588</v>
       </c>
       <c r="O28" s="81" t="s">
-        <v>2955</v>
+        <v>2954</v>
       </c>
       <c r="P28" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q28" s="58">
         <v>1</v>
@@ -42181,7 +42181,7 @@
       <c r="T28" s="59"/>
       <c r="U28" s="63"/>
       <c r="V28" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W28" s="58">
         <v>1</v>
@@ -42209,7 +42209,7 @@
         <v>621</v>
       </c>
       <c r="E29" s="48" t="s">
-        <v>2940</v>
+        <v>2939</v>
       </c>
       <c r="F29" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B29, prodcom_data[product], 0))</f>
@@ -42230,23 +42230,23 @@
         <v>2642</v>
       </c>
       <c r="K29" s="79" t="s">
-        <v>2941</v>
+        <v>2940</v>
       </c>
       <c r="L29" s="79">
         <v>86.09</v>
       </c>
       <c r="M29" s="80" t="s">
-        <v>2926</v>
+        <v>2925</v>
       </c>
       <c r="N29" s="72">
         <f>M29*Calculations!$C$37/L29</f>
         <v>0.55806713904053895</v>
       </c>
       <c r="O29" s="81" t="s">
-        <v>2942</v>
+        <v>2941</v>
       </c>
       <c r="P29" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q29" s="58">
         <v>1</v>
@@ -42256,7 +42256,7 @@
       <c r="T29" s="59"/>
       <c r="U29" s="63"/>
       <c r="V29" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W29" s="58">
         <v>1</v>
@@ -42305,23 +42305,23 @@
         <v>2642</v>
       </c>
       <c r="K30" s="79" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
       <c r="L30" s="79">
         <v>60.05</v>
       </c>
       <c r="M30" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N30" s="72">
         <f>M30*Calculations!$C$37/L30</f>
         <v>0.40003330557868444</v>
       </c>
       <c r="O30" s="81" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
       <c r="P30" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q30" s="58">
         <v>1</v>
@@ -42331,7 +42331,7 @@
       <c r="T30" s="59"/>
       <c r="U30" s="63"/>
       <c r="V30" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W30" s="58">
         <v>1</v>
@@ -42359,7 +42359,7 @@
         <v>474</v>
       </c>
       <c r="E31" s="48" t="s">
-        <v>2963</v>
+        <v>2962</v>
       </c>
       <c r="F31" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B31, prodcom_data[product], 0))</f>
@@ -42380,23 +42380,23 @@
         <v>2642</v>
       </c>
       <c r="K31" s="79" t="s">
-        <v>2964</v>
+        <v>2963</v>
       </c>
       <c r="L31" s="79">
         <v>44.05</v>
       </c>
       <c r="M31" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N31" s="72">
         <f>M31*Calculations!$C$37/L31</f>
         <v>0.54533484676503974</v>
       </c>
       <c r="O31" s="81" t="s">
-        <v>2965</v>
+        <v>2964</v>
       </c>
       <c r="P31" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q31" s="58">
         <v>1</v>
@@ -42406,7 +42406,7 @@
       <c r="T31" s="59"/>
       <c r="U31" s="63"/>
       <c r="V31" s="59" t="s">
-        <v>3045</v>
+        <v>3044</v>
       </c>
       <c r="W31" s="58">
         <v>1</v>
@@ -42434,7 +42434,7 @@
         <v>79</v>
       </c>
       <c r="E32" s="48" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
       <c r="F32" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B32, prodcom_data[product], 0))</f>
@@ -42455,23 +42455,23 @@
         <v>2642</v>
       </c>
       <c r="K32" s="79" t="s">
-        <v>2912</v>
+        <v>2911</v>
       </c>
       <c r="L32" s="79">
         <v>62.5</v>
       </c>
       <c r="M32" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N32" s="72">
         <f>M32*Calculations!$C$37/L32</f>
         <v>0.38435199999999997</v>
       </c>
       <c r="O32" s="81" t="s">
-        <v>2913</v>
+        <v>2912</v>
       </c>
       <c r="P32" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q32" s="58">
         <v>1</v>
@@ -42481,7 +42481,7 @@
       <c r="T32" s="59"/>
       <c r="U32" s="63"/>
       <c r="V32" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W32" s="58">
         <v>1</v>
@@ -42509,7 +42509,7 @@
         <v>294</v>
       </c>
       <c r="E33" s="48" t="s">
-        <v>2950</v>
+        <v>2949</v>
       </c>
       <c r="F33" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B33, prodcom_data[product], 0))</f>
@@ -42530,29 +42530,29 @@
         <v>2642</v>
       </c>
       <c r="K33" s="79" t="s">
-        <v>2951</v>
+        <v>2950</v>
       </c>
       <c r="L33" s="79">
         <v>93.13</v>
       </c>
       <c r="M33" s="80" t="s">
-        <v>2909</v>
+        <v>2908</v>
       </c>
       <c r="N33" s="72">
         <f>M33*Calculations!$C$37/L33</f>
         <v>0.77382153978309898</v>
       </c>
       <c r="O33" s="81" t="s">
-        <v>2952</v>
+        <v>2951</v>
       </c>
       <c r="P33" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q33" s="58">
         <v>0.8</v>
       </c>
       <c r="R33" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S33" s="61" cm="1">
         <f t="array" ref="S33">1-SUM(IF(ISNUMBER(P33:Q33), P33:Q33, 0))</f>
@@ -42561,13 +42561,13 @@
       <c r="T33" s="59"/>
       <c r="U33" s="63"/>
       <c r="V33" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W33" s="58">
         <v>0.8</v>
       </c>
       <c r="X33" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y33" s="61" cm="1">
         <f t="array" ref="Y33">1-SUM(IF(ISNUMBER(V33:W33), V33:W33, 0))</f>
@@ -42594,7 +42594,7 @@
         <v>603</v>
       </c>
       <c r="E34" s="48" t="s">
-        <v>2918</v>
+        <v>2917</v>
       </c>
       <c r="F34" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B34, prodcom_data[product], 0))</f>
@@ -42615,23 +42615,23 @@
         <v>2642</v>
       </c>
       <c r="K34" s="79" t="s">
-        <v>2919</v>
+        <v>2918</v>
       </c>
       <c r="L34" s="79">
         <v>222.24</v>
       </c>
       <c r="M34" s="80" t="s">
-        <v>2920</v>
+        <v>2919</v>
       </c>
       <c r="N34" s="72">
         <f>M34*Calculations!$C$37/L34</f>
         <v>0.64854211663066952</v>
       </c>
       <c r="O34" s="81" t="s">
-        <v>2921</v>
+        <v>2920</v>
       </c>
       <c r="P34" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q34" s="58">
         <v>1</v>
@@ -42641,7 +42641,7 @@
       <c r="T34" s="59"/>
       <c r="U34" s="63"/>
       <c r="V34" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W34" s="58">
         <v>1</v>
@@ -42669,7 +42669,7 @@
         <v>136</v>
       </c>
       <c r="E35" s="48" t="s">
-        <v>2984</v>
+        <v>2983</v>
       </c>
       <c r="F35" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B35, prodcom_data[product], 0))</f>
@@ -42690,29 +42690,29 @@
         <v>2642</v>
       </c>
       <c r="K35" s="79" t="s">
-        <v>2985</v>
+        <v>2984</v>
       </c>
       <c r="L35" s="79">
         <v>76.09</v>
       </c>
       <c r="M35" s="80" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="N35" s="72">
         <f>M35*Calculations!$C$37/L35</f>
         <v>0.47355762912340649</v>
       </c>
       <c r="O35" s="81" t="s">
-        <v>2986</v>
+        <v>2985</v>
       </c>
       <c r="P35" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q35" s="58">
         <v>0.95</v>
       </c>
       <c r="R35" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S35" s="61" cm="1">
         <f t="array" ref="S35">1-SUM(IF(ISNUMBER(P35:Q35), P35:Q35, 0))</f>
@@ -42721,13 +42721,13 @@
       <c r="T35" s="59"/>
       <c r="U35" s="63"/>
       <c r="V35" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W35" s="58">
         <v>0.95</v>
       </c>
       <c r="X35" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y35" s="61" cm="1">
         <f t="array" ref="Y35">1-SUM(IF(ISNUMBER(V35:W35), V35:W35, 0))</f>
@@ -42754,7 +42754,7 @@
         <v>558</v>
       </c>
       <c r="E36" s="48" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
       <c r="F36" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B36, prodcom_data[product], 0))</f>
@@ -42775,23 +42775,23 @@
         <v>2642</v>
       </c>
       <c r="K36" s="79" t="s">
-        <v>2959</v>
+        <v>2958</v>
       </c>
       <c r="L36" s="79">
         <v>211.3</v>
       </c>
       <c r="M36" s="80" t="s">
-        <v>2960</v>
+        <v>2959</v>
       </c>
       <c r="N36" s="72">
         <f>M36*Calculations!$C$37/L36</f>
         <v>0.85265026029342161</v>
       </c>
       <c r="O36" s="81" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
       <c r="P36" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q36" s="58">
         <v>1</v>
@@ -42801,7 +42801,7 @@
       <c r="T36" s="59"/>
       <c r="U36" s="63"/>
       <c r="V36" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W36" s="58">
         <v>1</v>
@@ -42829,7 +42829,7 @@
         <v>47</v>
       </c>
       <c r="E37" s="48" t="s">
-        <v>2993</v>
+        <v>2992</v>
       </c>
       <c r="F37" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B37, prodcom_data[product], 0))</f>
@@ -42850,29 +42850,29 @@
         <v>2642</v>
       </c>
       <c r="K37" s="79" t="s">
-        <v>2981</v>
+        <v>2980</v>
       </c>
       <c r="L37" s="79">
         <v>106.16</v>
       </c>
       <c r="M37" s="80" t="s">
-        <v>2916</v>
+        <v>2915</v>
       </c>
       <c r="N37" s="72">
         <f>M37*Calculations!$C$37/L37</f>
         <v>0.90512434061793512</v>
       </c>
       <c r="O37" s="81" t="s">
-        <v>2994</v>
+        <v>2993</v>
       </c>
       <c r="P37" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q37" s="58">
         <v>0.97</v>
       </c>
       <c r="R37" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S37" s="61" cm="1">
         <f t="array" ref="S37">1-SUM(IF(ISNUMBER(P37:Q37), P37:Q37, 0))</f>
@@ -42881,13 +42881,13 @@
       <c r="T37" s="59"/>
       <c r="U37" s="63"/>
       <c r="V37" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W37" s="58">
         <v>0.97</v>
       </c>
       <c r="X37" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y37" s="61" cm="1">
         <f t="array" ref="Y37">1-SUM(IF(ISNUMBER(V37:W37), V37:W37, 0))</f>
@@ -42914,7 +42914,7 @@
         <v>570</v>
       </c>
       <c r="E38" s="48" t="s">
-        <v>2911</v>
+        <v>2910</v>
       </c>
       <c r="F38" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B38, prodcom_data[product], 0))</f>
@@ -42935,29 +42935,29 @@
         <v>2642</v>
       </c>
       <c r="K38" s="79" t="s">
-        <v>2912</v>
+        <v>2911</v>
       </c>
       <c r="L38" s="79">
         <v>62.5</v>
       </c>
       <c r="M38" s="80" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="N38" s="72">
         <f>M38*Calculations!$C$37/L38</f>
         <v>0.38435199999999997</v>
       </c>
       <c r="O38" s="81" t="s">
-        <v>2913</v>
+        <v>2912</v>
       </c>
       <c r="P38" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q38" s="58">
         <v>0.98</v>
       </c>
       <c r="R38" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S38" s="61" cm="1">
         <f t="array" ref="S38">1-SUM(IF(ISNUMBER(P38:Q38), P38:Q38, 0))</f>
@@ -42966,13 +42966,13 @@
       <c r="T38" s="59"/>
       <c r="U38" s="63"/>
       <c r="V38" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W38" s="58">
         <v>0.98</v>
       </c>
       <c r="X38" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y38" s="61" cm="1">
         <f t="array" ref="Y38">1-SUM(IF(ISNUMBER(V38:W38), V38:W38, 0))</f>
@@ -43020,29 +43020,29 @@
         <v>2642</v>
       </c>
       <c r="K39" s="79" t="s">
-        <v>2974</v>
+        <v>2973</v>
       </c>
       <c r="L39" s="79">
         <v>120.19</v>
       </c>
       <c r="M39" s="80" t="s">
-        <v>2975</v>
+        <v>2974</v>
       </c>
       <c r="N39" s="72">
         <f>M39*Calculations!$C$37/L39</f>
         <v>0.89940094849821106</v>
       </c>
       <c r="O39" s="81" t="s">
-        <v>2976</v>
+        <v>2975</v>
       </c>
       <c r="P39" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q39" s="58">
         <v>0.94</v>
       </c>
       <c r="R39" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S39" s="61" cm="1">
         <f t="array" ref="S39">1-SUM(IF(ISNUMBER(P39:Q39), P39:Q39, 0))</f>
@@ -43051,13 +43051,13 @@
       <c r="T39" s="59"/>
       <c r="U39" s="63"/>
       <c r="V39" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W39" s="58">
         <v>0.94</v>
       </c>
       <c r="X39" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y39" s="61" cm="1">
         <f t="array" ref="Y39">1-SUM(IF(ISNUMBER(V39:W39), V39:W39, 0))</f>
@@ -43105,23 +43105,23 @@
         <v>2642</v>
       </c>
       <c r="K40" s="79" t="s">
-        <v>2999</v>
+        <v>2998</v>
       </c>
       <c r="L40" s="79">
         <v>53.06</v>
       </c>
       <c r="M40" s="80" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="N40" s="72">
         <f>M40*Calculations!$C$37/L40</f>
         <v>0.67909913305691672</v>
       </c>
       <c r="O40" s="81" t="s">
-        <v>3000</v>
+        <v>2999</v>
       </c>
       <c r="P40" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q40" s="58">
         <v>1</v>
@@ -43131,7 +43131,7 @@
       <c r="T40" s="59"/>
       <c r="U40" s="63"/>
       <c r="V40" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W40" s="58">
         <v>1</v>
@@ -43180,23 +43180,23 @@
         <v>2642</v>
       </c>
       <c r="K41" s="79" t="s">
-        <v>2977</v>
+        <v>2976</v>
       </c>
       <c r="L41" s="79">
         <v>84.16</v>
       </c>
       <c r="M41" s="80" t="s">
-        <v>2909</v>
+        <v>2908</v>
       </c>
       <c r="N41" s="72">
         <f>M41*Calculations!$C$37/L41</f>
         <v>0.85629752851711038</v>
       </c>
       <c r="O41" s="81" t="s">
-        <v>2978</v>
+        <v>2977</v>
       </c>
       <c r="P41" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q41" s="58">
         <v>1</v>
@@ -43206,7 +43206,7 @@
       <c r="T41" s="59"/>
       <c r="U41" s="63"/>
       <c r="V41" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W41" s="58">
         <v>1</v>
@@ -43255,23 +43255,23 @@
         <v>2642</v>
       </c>
       <c r="K42" s="79" t="s">
-        <v>2979</v>
+        <v>2978</v>
       </c>
       <c r="L42" s="79">
         <v>146.13999999999999</v>
       </c>
       <c r="M42" s="80" t="s">
-        <v>2909</v>
+        <v>2908</v>
       </c>
       <c r="N42" s="72">
         <f>M42*Calculations!$C$37/L42</f>
         <v>0.49312987546188591</v>
       </c>
       <c r="O42" s="81" t="s">
-        <v>2980</v>
+        <v>2979</v>
       </c>
       <c r="P42" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q42" s="58">
         <v>1</v>
@@ -43281,7 +43281,7 @@
       <c r="T42" s="59"/>
       <c r="U42" s="63"/>
       <c r="V42" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W42" s="58">
         <v>1</v>
@@ -43309,7 +43309,7 @@
         <v>115</v>
       </c>
       <c r="E43" s="48" t="s">
-        <v>2971</v>
+        <v>2970</v>
       </c>
       <c r="F43" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B43, prodcom_data[product], 0))</f>
@@ -43330,29 +43330,29 @@
         <v>2687</v>
       </c>
       <c r="K43" s="79" t="s">
-        <v>2972</v>
+        <v>2971</v>
       </c>
       <c r="L43" s="79">
         <v>60.1</v>
       </c>
       <c r="M43" s="80" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="N43" s="72">
         <f>M43*Calculations!$C$37/L43</f>
         <v>0.59955074875207992</v>
       </c>
       <c r="O43" s="81" t="s">
-        <v>2973</v>
+        <v>2972</v>
       </c>
       <c r="P43" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q43" s="58">
         <v>0.82</v>
       </c>
       <c r="R43" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S43" s="61" cm="1">
         <f t="array" ref="S43">1-SUM(IF(ISNUMBER(P43:Q43), P43:Q43, 0))</f>
@@ -43361,13 +43361,13 @@
       <c r="T43" s="59"/>
       <c r="U43" s="63"/>
       <c r="V43" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W43" s="58">
         <v>0.82</v>
       </c>
       <c r="X43" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y43" s="61" cm="1">
         <f t="array" ref="Y43">1-SUM(IF(ISNUMBER(V43:W43), V43:W43, 0))</f>
@@ -43415,23 +43415,23 @@
         <v>2642</v>
       </c>
       <c r="K44" s="79" t="s">
-        <v>2981</v>
+        <v>2980</v>
       </c>
       <c r="L44" s="79">
         <v>106.16</v>
       </c>
       <c r="M44" s="80" t="s">
-        <v>2916</v>
+        <v>2915</v>
       </c>
       <c r="N44" s="72">
         <f>M44*Calculations!$C$37/L44</f>
         <v>0.90512434061793512</v>
       </c>
       <c r="O44" s="81" t="s">
-        <v>2983</v>
+        <v>2982</v>
       </c>
       <c r="P44" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q44" s="58">
         <v>1</v>
@@ -43441,7 +43441,7 @@
       <c r="T44" s="59"/>
       <c r="U44" s="63"/>
       <c r="V44" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W44" s="58">
         <v>1</v>
@@ -43490,29 +43490,29 @@
         <v>2689</v>
       </c>
       <c r="K45" s="79" t="s">
-        <v>2969</v>
+        <v>2968</v>
       </c>
       <c r="L45" s="79">
         <v>128.16900000000001</v>
       </c>
       <c r="M45" s="80" t="s">
-        <v>2948</v>
+        <v>2947</v>
       </c>
       <c r="N45" s="72">
         <f>M45*Calculations!$C$37/L45</f>
         <v>0.6559854567016985</v>
       </c>
       <c r="O45" s="81" t="s">
-        <v>2970</v>
+        <v>2969</v>
       </c>
       <c r="P45" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q45" s="58">
         <v>0.72</v>
       </c>
       <c r="R45" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S45" s="61" cm="1">
         <f t="array" ref="S45">1-SUM(IF(ISNUMBER(P45:Q45), P45:Q45, 0))</f>
@@ -43521,13 +43521,13 @@
       <c r="T45" s="59"/>
       <c r="U45" s="63"/>
       <c r="V45" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W45" s="58">
         <v>0.72</v>
       </c>
       <c r="X45" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y45" s="61" cm="1">
         <f t="array" ref="Y45">1-SUM(IF(ISNUMBER(V45:W45), V45:W45, 0))</f>
@@ -43554,7 +43554,7 @@
         <v>543</v>
       </c>
       <c r="E46" s="48" t="s">
-        <v>2966</v>
+        <v>2965</v>
       </c>
       <c r="F46" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B46, prodcom_data[product], 0))</f>
@@ -43575,29 +43575,29 @@
         <v>2642</v>
       </c>
       <c r="K46" s="79" t="s">
-        <v>2967</v>
+        <v>2966</v>
       </c>
       <c r="L46" s="79">
         <v>114.14</v>
       </c>
       <c r="M46" s="80" t="s">
-        <v>2909</v>
+        <v>2908</v>
       </c>
       <c r="N46" s="72">
         <f>M46*Calculations!$C$37/L46</f>
         <v>0.63138251270369727</v>
       </c>
       <c r="O46" s="81" t="s">
-        <v>2968</v>
+        <v>2967</v>
       </c>
       <c r="P46" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q46" s="58">
         <v>0.87</v>
       </c>
       <c r="R46" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S46" s="61" cm="1">
         <f t="array" ref="S46">1-SUM(IF(ISNUMBER(P46:Q46), P46:Q46, 0))</f>
@@ -43606,13 +43606,13 @@
       <c r="T46" s="59"/>
       <c r="U46" s="63"/>
       <c r="V46" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W46" s="58">
         <v>0.87</v>
       </c>
       <c r="X46" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y46" s="61" cm="1">
         <f t="array" ref="Y46">1-SUM(IF(ISNUMBER(V46:W46), V46:W46, 0))</f>
@@ -43639,7 +43639,7 @@
         <v>118</v>
       </c>
       <c r="E47" s="48" t="s">
-        <v>2987</v>
+        <v>2986</v>
       </c>
       <c r="F47" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B47, prodcom_data[product], 0))</f>
@@ -43660,23 +43660,23 @@
         <v>2642</v>
       </c>
       <c r="K47" s="79" t="s">
-        <v>2988</v>
+        <v>2987</v>
       </c>
       <c r="L47" s="79">
         <v>74.12</v>
       </c>
       <c r="M47" s="80" t="s">
-        <v>2926</v>
+        <v>2925</v>
       </c>
       <c r="N47" s="72">
         <f>M47*Calculations!$C$37/L47</f>
         <v>0.64819212088505118</v>
       </c>
       <c r="O47" s="81" t="s">
-        <v>2989</v>
+        <v>2988</v>
       </c>
       <c r="P47" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q47" s="58">
         <v>1</v>
@@ -43686,7 +43686,7 @@
       <c r="T47" s="59"/>
       <c r="U47" s="63"/>
       <c r="V47" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W47" s="58">
         <v>1</v>
@@ -43714,7 +43714,7 @@
         <v>285</v>
       </c>
       <c r="E48" s="48" t="s">
-        <v>2990</v>
+        <v>2989</v>
       </c>
       <c r="F48" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B48, prodcom_data[product], 0))</f>
@@ -43735,29 +43735,29 @@
         <v>2693</v>
       </c>
       <c r="K48" s="79" t="s">
-        <v>2991</v>
+        <v>2990</v>
       </c>
       <c r="L48" s="79">
         <v>116.2</v>
       </c>
       <c r="M48" s="80" t="s">
-        <v>2909</v>
+        <v>2908</v>
       </c>
       <c r="N48" s="72">
         <f>M48*Calculations!$C$37/L48</f>
         <v>0.6201893287435456</v>
       </c>
       <c r="O48" s="81" t="s">
-        <v>2992</v>
+        <v>2991</v>
       </c>
       <c r="P48" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q48" s="58">
         <v>0.91</v>
       </c>
       <c r="R48" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S48" s="61" cm="1">
         <f t="array" ref="S48">1-SUM(IF(ISNUMBER(P48:Q48), P48:Q48, 0))</f>
@@ -43766,13 +43766,13 @@
       <c r="T48" s="59"/>
       <c r="U48" s="63"/>
       <c r="V48" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W48" s="58">
         <v>0.91</v>
       </c>
       <c r="X48" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y48" s="61" cm="1">
         <f t="array" ref="Y48">1-SUM(IF(ISNUMBER(V48:W48), V48:W48, 0))</f>
@@ -43820,23 +43820,23 @@
         <v>2642</v>
       </c>
       <c r="K49" s="79" t="s">
-        <v>3005</v>
+        <v>3004</v>
       </c>
       <c r="L49" s="79">
         <v>88.11</v>
       </c>
       <c r="M49" s="80" t="s">
-        <v>2926</v>
+        <v>2925</v>
       </c>
       <c r="N49" s="72">
         <f>M49*Calculations!$C$37/L49</f>
         <v>0.54527295426171829</v>
       </c>
       <c r="O49" s="81" t="s">
-        <v>3006</v>
+        <v>3005</v>
       </c>
       <c r="P49" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="Q49" s="58">
         <v>1</v>
@@ -43846,7 +43846,7 @@
       <c r="T49" s="59"/>
       <c r="U49" s="63"/>
       <c r="V49" s="59" t="s">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="W49" s="58">
         <v>1</v>
@@ -43874,7 +43874,7 @@
         <v>582</v>
       </c>
       <c r="E50" s="48" t="s">
-        <v>3001</v>
+        <v>3000</v>
       </c>
       <c r="F50" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B50, prodcom_data[product], 0))</f>
@@ -43889,26 +43889,26 @@
         <v>0.59226283959165005</v>
       </c>
       <c r="I50" s="51" t="s">
-        <v>3002</v>
+        <v>3001</v>
       </c>
       <c r="J50" s="49" t="s">
         <v>2695</v>
       </c>
       <c r="K50" s="79" t="s">
-        <v>3003</v>
+        <v>3002</v>
       </c>
       <c r="L50" s="79">
         <v>30.026</v>
       </c>
       <c r="M50" s="80" t="s">
-        <v>2906</v>
+        <v>2905</v>
       </c>
       <c r="N50" s="72">
         <f>M50*Calculations!$C$37/L50</f>
         <v>0.40001998268167588</v>
       </c>
       <c r="O50" s="81" t="s">
-        <v>3004</v>
+        <v>3003</v>
       </c>
       <c r="P50" s="59"/>
       <c r="Q50" s="60"/>
@@ -43941,7 +43941,7 @@
         <v>460</v>
       </c>
       <c r="E51" s="48" t="s">
-        <v>3007</v>
+        <v>3006</v>
       </c>
       <c r="F51" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B51, prodcom_data[product], 0))</f>
@@ -43962,29 +43962,29 @@
         <v>2642</v>
       </c>
       <c r="K51" s="79" t="s">
-        <v>3008</v>
+        <v>3007</v>
       </c>
       <c r="L51" s="79">
         <v>106.12</v>
       </c>
       <c r="M51" s="80" t="s">
-        <v>2926</v>
+        <v>2925</v>
       </c>
       <c r="N51" s="72">
         <f>M51*Calculations!$C$37/L51</f>
         <v>0.45273275537127777</v>
       </c>
       <c r="O51" s="81" t="s">
-        <v>3009</v>
+        <v>3008</v>
       </c>
       <c r="P51" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q51" s="58">
         <v>0.21</v>
       </c>
       <c r="R51" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S51" s="61" cm="1">
         <f t="array" ref="S51">1-SUM(IF(ISNUMBER(P51:Q51), P51:Q51, 0))</f>
@@ -43993,13 +43993,13 @@
       <c r="T51" s="59"/>
       <c r="U51" s="63"/>
       <c r="V51" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W51" s="58">
         <v>0.21</v>
       </c>
       <c r="X51" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y51" s="61" cm="1">
         <f t="array" ref="Y51">1-SUM(IF(ISNUMBER(V51:W51), V51:W51, 0))</f>
@@ -44026,7 +44026,7 @@
         <v>227</v>
       </c>
       <c r="E52" s="48" t="s">
-        <v>2995</v>
+        <v>2994</v>
       </c>
       <c r="F52" s="56">
         <f>INDEX(prodcom_data[PRODQNT + IMPQNT - EU27 - 2022], MATCH(B52, prodcom_data[product], 0))</f>
@@ -44047,29 +44047,29 @@
         <v>2698</v>
       </c>
       <c r="K52" s="79" t="s">
-        <v>2996</v>
+        <v>2995</v>
       </c>
       <c r="L52" s="79">
         <v>100.12</v>
       </c>
       <c r="M52" s="80" t="s">
-        <v>2997</v>
+        <v>2996</v>
       </c>
       <c r="N52" s="72">
         <f>M52*Calculations!$C$37/L52</f>
         <v>0.59983020375549334</v>
       </c>
       <c r="O52" s="81" t="s">
-        <v>2998</v>
+        <v>2997</v>
       </c>
       <c r="P52" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q52" s="58">
         <v>0.35</v>
       </c>
       <c r="R52" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S52" s="61" cm="1">
         <f t="array" ref="S52">1-SUM(IF(ISNUMBER(P52:Q52), P52:Q52, 0))</f>
@@ -44078,13 +44078,13 @@
       <c r="T52" s="59"/>
       <c r="U52" s="63"/>
       <c r="V52" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W52" s="58">
         <v>0.35</v>
       </c>
       <c r="X52" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y52" s="61" cm="1">
         <f t="array" ref="Y52">1-SUM(IF(ISNUMBER(V52:W52), V52:W52, 0))</f>
@@ -44132,29 +44132,29 @@
         <v>2642</v>
       </c>
       <c r="K53" s="79" t="s">
-        <v>2981</v>
+        <v>2980</v>
       </c>
       <c r="L53" s="79">
         <v>106.16</v>
       </c>
       <c r="M53" s="80" t="s">
-        <v>2916</v>
+        <v>2915</v>
       </c>
       <c r="N53" s="72">
         <f>M53*Calculations!$C$37/L53</f>
         <v>0.90512434061793512</v>
       </c>
       <c r="O53" s="81" t="s">
-        <v>3010</v>
+        <v>3009</v>
       </c>
       <c r="P53" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q53" s="58">
         <v>0.51</v>
       </c>
       <c r="R53" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S53" s="61" cm="1">
         <f t="array" ref="S53">1-SUM(IF(ISNUMBER(P53:Q53), P53:Q53, 0))</f>
@@ -44163,13 +44163,13 @@
       <c r="T53" s="59"/>
       <c r="U53" s="63"/>
       <c r="V53" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W53" s="58">
         <v>0.51</v>
       </c>
       <c r="X53" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y53" s="61" cm="1">
         <f t="array" ref="Y53">1-SUM(IF(ISNUMBER(V53:W53), V53:W53, 0))</f>
@@ -44193,10 +44193,10 @@
         <v>2829</v>
       </c>
       <c r="D54" s="52" t="s">
+        <v>3010</v>
+      </c>
+      <c r="E54" s="48" t="s">
         <v>3011</v>
-      </c>
-      <c r="E54" s="48" t="s">
-        <v>3012</v>
       </c>
       <c r="F54" s="56">
         <f>Calculations!C32*(Calculations!C29/SUM(Calculations!$C$28:$C$29))</f>
@@ -44211,35 +44211,35 @@
         <v>0.88632047658515611</v>
       </c>
       <c r="I54" s="48" t="s">
-        <v>3013</v>
+        <v>3012</v>
       </c>
       <c r="J54" s="49" t="s">
         <v>2671</v>
       </c>
       <c r="K54" s="79" t="s">
-        <v>3014</v>
+        <v>3013</v>
       </c>
       <c r="L54" s="79">
         <v>174.16</v>
       </c>
       <c r="M54" s="80" t="s">
-        <v>2975</v>
+        <v>2974</v>
       </c>
       <c r="N54" s="72">
         <f>M54*Calculations!$C$37/L54</f>
         <v>0.6206878732200275</v>
       </c>
       <c r="O54" s="81" t="s">
-        <v>3015</v>
+        <v>3014</v>
       </c>
       <c r="P54" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q54" s="58">
         <v>0.88</v>
       </c>
       <c r="R54" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S54" s="61" cm="1">
         <f t="array" ref="S54">1-SUM(IF(ISNUMBER(P54:Q54), P54:Q54, 0))</f>
@@ -44248,13 +44248,13 @@
       <c r="T54" s="59"/>
       <c r="U54" s="63"/>
       <c r="V54" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W54" s="58">
         <v>0.88</v>
       </c>
       <c r="X54" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y54" s="61" cm="1">
         <f t="array" ref="Y54">1-SUM(IF(ISNUMBER(V54:W54), V54:W54, 0))</f>
@@ -44278,10 +44278,10 @@
         <v>2829</v>
       </c>
       <c r="D55" s="52" t="s">
+        <v>3015</v>
+      </c>
+      <c r="E55" s="48" t="s">
         <v>3016</v>
-      </c>
-      <c r="E55" s="48" t="s">
-        <v>3017</v>
       </c>
       <c r="F55" s="56">
         <f>Calculations!C32*(Calculations!C28/SUM(Calculations!$C$28:$C$29))</f>
@@ -44296,35 +44296,35 @@
         <v>0.88632047658515611</v>
       </c>
       <c r="I55" s="48" t="s">
-        <v>3018</v>
+        <v>3017</v>
       </c>
       <c r="J55" s="49" t="s">
         <v>2671</v>
       </c>
       <c r="K55" s="79" t="s">
-        <v>3019</v>
+        <v>3018</v>
       </c>
       <c r="L55" s="79">
         <v>250.25</v>
       </c>
       <c r="M55" s="80" t="s">
-        <v>2960</v>
+        <v>2959</v>
       </c>
       <c r="N55" s="72">
         <f>M55*Calculations!$C$37/L55</f>
         <v>0.71994005994005994</v>
       </c>
       <c r="O55" s="81" t="s">
-        <v>3020</v>
+        <v>3019</v>
       </c>
       <c r="P55" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q55" s="58">
         <v>0.88</v>
       </c>
       <c r="R55" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S55" s="61" cm="1">
         <f t="array" ref="S55">1-SUM(IF(ISNUMBER(P55:Q55), P55:Q55, 0))</f>
@@ -44333,13 +44333,13 @@
       <c r="T55" s="59"/>
       <c r="U55" s="63"/>
       <c r="V55" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W55" s="58">
         <v>0.88</v>
       </c>
       <c r="X55" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y55" s="61" cm="1">
         <f t="array" ref="Y55">1-SUM(IF(ISNUMBER(V55:W55), V55:W55, 0))</f>
@@ -44363,10 +44363,10 @@
         <v>2819</v>
       </c>
       <c r="D56" s="52" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E56" s="48" t="s">
         <v>3021</v>
-      </c>
-      <c r="E56" s="48" t="s">
-        <v>3022</v>
       </c>
       <c r="F56" s="56">
         <f>Calculations!C6*(Calculations!C24/(Calculations!C15+Calculations!C24))</f>
@@ -44381,35 +44381,35 @@
         <v>0.87748442629671652</v>
       </c>
       <c r="I56" s="48" t="s">
-        <v>3023</v>
+        <v>3022</v>
       </c>
       <c r="J56" s="49" t="s">
         <v>2661</v>
       </c>
       <c r="K56" s="79" t="s">
-        <v>3024</v>
+        <v>3023</v>
       </c>
       <c r="L56" s="79">
         <v>224.3</v>
       </c>
       <c r="M56" s="80" t="s">
-        <v>2920</v>
+        <v>2919</v>
       </c>
       <c r="N56" s="72">
         <f>M56*Calculations!$C$37/L56</f>
         <v>0.64258582255907271</v>
       </c>
       <c r="O56" s="81" t="s">
-        <v>3025</v>
+        <v>3024</v>
       </c>
       <c r="P56" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q56" s="58">
         <v>0.91</v>
       </c>
       <c r="R56" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S56" s="61" cm="1">
         <f t="array" ref="S56">1-SUM(IF(ISNUMBER(P56:Q56), P56:Q56, 0))</f>
@@ -44418,13 +44418,13 @@
       <c r="T56" s="59"/>
       <c r="U56" s="63"/>
       <c r="V56" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W56" s="58">
         <v>0.91</v>
       </c>
       <c r="X56" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y56" s="61" cm="1">
         <f t="array" ref="Y56">1-SUM(IF(ISNUMBER(V56:W56), V56:W56, 0))</f>
@@ -44448,10 +44448,10 @@
         <v>2819</v>
       </c>
       <c r="D57" s="52" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E57" s="48" t="s">
         <v>3026</v>
-      </c>
-      <c r="E57" s="48" t="s">
-        <v>3027</v>
       </c>
       <c r="F57" s="56">
         <f>Calculations!C6*(Calculations!C15/(Calculations!C15+Calculations!C24))</f>
@@ -44466,35 +44466,35 @@
         <v>0.87748442629671652</v>
       </c>
       <c r="I57" s="48" t="s">
-        <v>3028</v>
+        <v>3027</v>
       </c>
       <c r="J57" s="49" t="s">
         <v>2661</v>
       </c>
       <c r="K57" s="79" t="s">
-        <v>3029</v>
+        <v>3028</v>
       </c>
       <c r="L57" s="79">
         <v>582.79999999999995</v>
       </c>
       <c r="M57" s="80" t="s">
-        <v>3030</v>
+        <v>3029</v>
       </c>
       <c r="N57" s="72">
         <f>M57*Calculations!$C$37/L57</f>
         <v>0.61827385037748805</v>
       </c>
       <c r="O57" s="81" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="P57" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="Q57" s="58">
         <v>0.91</v>
       </c>
       <c r="R57" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="S57" s="61" cm="1">
         <f t="array" ref="S57">1-SUM(IF(ISNUMBER(P57:Q57), P57:Q57, 0))</f>
@@ -44503,13 +44503,13 @@
       <c r="T57" s="59"/>
       <c r="U57" s="63"/>
       <c r="V57" s="59" t="s">
-        <v>3037</v>
+        <v>3036</v>
       </c>
       <c r="W57" s="58">
         <v>0.91</v>
       </c>
       <c r="X57" s="59" t="s">
-        <v>3044</v>
+        <v>3043</v>
       </c>
       <c r="Y57" s="61" cm="1">
         <f t="array" ref="Y57">1-SUM(IF(ISNUMBER(V57:W57), V57:W57, 0))</f>
@@ -44550,10 +44550,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="50" t="s">
+        <v>3058</v>
+      </c>
+      <c r="B1" t="s">
         <v>3059</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3060</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Update figure post-processing and update Step 4 Excel with new data
</commit_message>
<xml_diff>
--- a/Article_data/Step 3 results from Prodcom data manipulations.xlsx
+++ b/Article_data/Step 3 results from Prodcom data manipulations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nicolas\projects\202604-paper-1-supplementary-code\Article_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A660D838-64B7-4AB0-934B-596014D9CB26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{446257C7-A827-451F-A9E9-D43B6D007B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28935" yWindow="-45" windowWidth="29070" windowHeight="15750" tabRatio="570" activeTab="3" xr2:uid="{EE4678C9-3BCB-4D41-A2DA-6855614353C7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="570" xr2:uid="{EE4678C9-3BCB-4D41-A2DA-6855614353C7}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -54,7 +54,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Nicolas Lienart:</t>
         </r>
@@ -63,7 +63,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Saudi Arabia and South Korea</t>
@@ -78,7 +78,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Nicolas Lienart:</t>
         </r>
@@ -87,7 +87,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 United States + Mexico</t>
@@ -9465,7 +9465,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9610,19 +9610,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="9">
@@ -10038,14 +10025,14 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="15">
@@ -40482,10 +40469,10 @@
       </c>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="F7" s="96" t="s">
+      <c r="F7" s="98" t="s">
         <v>705</v>
       </c>
-      <c r="G7" s="96"/>
+      <c r="G7" s="98"/>
       <c r="I7" s="47" t="s">
         <v>3074</v>
       </c>
@@ -40610,7 +40597,7 @@
         <f>F9/1000000000</f>
         <v>11.059816493</v>
       </c>
-      <c r="H9" s="97">
+      <c r="H9" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B9, prodcom_data[product], 0))</f>
         <v>0.86402104863567564</v>
       </c>
@@ -40695,7 +40682,7 @@
         <f t="shared" ref="G10:G65" si="0">F10/1000000000</f>
         <v>10.337493766</v>
       </c>
-      <c r="H10" s="97">
+      <c r="H10" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B10, prodcom_data[product], 0))</f>
         <v>0.87904863332422545</v>
       </c>
@@ -40787,7 +40774,7 @@
         <f t="shared" si="0"/>
         <v>9.0817412019999999</v>
       </c>
-      <c r="H11" s="97">
+      <c r="H11" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B11, prodcom_data[product], 0))</f>
         <v>0.94409418582769256</v>
       </c>
@@ -40880,7 +40867,7 @@
         <f t="shared" si="0"/>
         <v>7.6288794710000003</v>
       </c>
-      <c r="H12" s="97">
+      <c r="H12" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B12, prodcom_data[product], 0))</f>
         <v>0.78369292184089345</v>
       </c>
@@ -40964,7 +40951,7 @@
         <f t="shared" si="0"/>
         <v>6.9047320579999996</v>
       </c>
-      <c r="H13" s="97">
+      <c r="H13" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B13, prodcom_data[product], 0))</f>
         <v>0.14193164800139446</v>
       </c>
@@ -41065,7 +41052,7 @@
         <f t="shared" si="0"/>
         <v>6.2344760670000001</v>
       </c>
-      <c r="H14" s="97">
+      <c r="H14" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B14, prodcom_data[product], 0))</f>
         <v>0.88287081478020857</v>
       </c>
@@ -41150,7 +41137,7 @@
         <f t="shared" si="0"/>
         <v>5.008047468</v>
       </c>
-      <c r="H15" s="97">
+      <c r="H15" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B15, prodcom_data[product], 0))</f>
         <v>0.89272188364169869</v>
       </c>
@@ -41240,7 +41227,7 @@
         <f t="shared" si="0"/>
         <v>4.4742138760000003</v>
       </c>
-      <c r="H16" s="97">
+      <c r="H16" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B16, prodcom_data[product], 0))</f>
         <v>0.7961067883023123</v>
       </c>
@@ -41324,7 +41311,7 @@
         <f t="shared" si="0"/>
         <v>4.2387100530000001</v>
       </c>
-      <c r="H17" s="97">
+      <c r="H17" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B17, prodcom_data[product], 0))</f>
         <v>0.8225375065540016</v>
       </c>
@@ -41399,7 +41386,7 @@
         <f t="shared" si="0"/>
         <v>3.6279763919999999</v>
       </c>
-      <c r="H18" s="97">
+      <c r="H18" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B18, prodcom_data[product], 0))</f>
         <v>0.82690725513409014</v>
       </c>
@@ -41492,7 +41479,7 @@
         <f t="shared" si="0"/>
         <v>3.4912837350000001</v>
       </c>
-      <c r="H19" s="97">
+      <c r="H19" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B19, prodcom_data[product], 0))</f>
         <v>0.80199726304971886</v>
       </c>
@@ -41567,7 +41554,7 @@
         <f t="shared" si="0"/>
         <v>3.34918497</v>
       </c>
-      <c r="H20" s="97">
+      <c r="H20" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B20, prodcom_data[product], 0))</f>
         <v>0.6568762309953875</v>
       </c>
@@ -41642,7 +41629,7 @@
         <f t="shared" si="0"/>
         <v>2.8089402570000002</v>
       </c>
-      <c r="H21" s="97">
+      <c r="H21" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B21, prodcom_data[product], 0))</f>
         <v>0.9968172135460267</v>
       </c>
@@ -41717,7 +41704,7 @@
         <f t="shared" si="0"/>
         <v>2.0000466659999998</v>
       </c>
-      <c r="H22" s="97">
+      <c r="H22" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B22, prodcom_data[product], 0))</f>
         <v>0.99997666754441616</v>
       </c>
@@ -41792,7 +41779,7 @@
         <f t="shared" si="0"/>
         <v>1.8640651770000001</v>
       </c>
-      <c r="H23" s="97">
+      <c r="H23" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B23, prodcom_data[product], 0))</f>
         <v>0.88707249478326589</v>
       </c>
@@ -41872,7 +41859,7 @@
         <f t="shared" si="0"/>
         <v>1.7957479670000001</v>
       </c>
-      <c r="H24" s="97">
+      <c r="H24" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B24, prodcom_data[product], 0))</f>
         <v>0.55687101886052137</v>
       </c>
@@ -41957,7 +41944,7 @@
         <f t="shared" si="0"/>
         <v>1.650938177</v>
       </c>
-      <c r="H25" s="97">
+      <c r="H25" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B25, prodcom_data[product], 0))</f>
         <v>0.98168669522505081</v>
       </c>
@@ -42041,7 +42028,7 @@
         <f t="shared" si="0"/>
         <v>1.592476459</v>
       </c>
-      <c r="H26" s="97">
+      <c r="H26" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B26, prodcom_data[product], 0))</f>
         <v>0.93163807390386044</v>
       </c>
@@ -42116,7 +42103,7 @@
         <f t="shared" si="0"/>
         <v>1.2029393820000001</v>
       </c>
-      <c r="H27" s="97">
+      <c r="H27" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B27, prodcom_data[product], 0))</f>
         <v>0.7564803460728331</v>
       </c>
@@ -42201,7 +42188,7 @@
         <f t="shared" si="0"/>
         <v>1.191905947</v>
       </c>
-      <c r="H28" s="97">
+      <c r="H28" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B28, prodcom_data[product], 0))</f>
         <v>0.46597635861951109</v>
       </c>
@@ -42286,7 +42273,7 @@
         <f t="shared" si="0"/>
         <v>1.1203816150000001</v>
       </c>
-      <c r="H29" s="97">
+      <c r="H29" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B29, prodcom_data[product], 0))</f>
         <v>0.97878773028598831</v>
       </c>
@@ -42361,7 +42348,7 @@
         <f t="shared" si="0"/>
         <v>1.0908528070000001</v>
       </c>
-      <c r="H30" s="97">
+      <c r="H30" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B30, prodcom_data[product], 0))</f>
         <v>0.92846915963429333</v>
       </c>
@@ -42446,7 +42433,7 @@
         <f t="shared" si="0"/>
         <v>0.931200527</v>
       </c>
-      <c r="H31" s="97">
+      <c r="H31" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B31, prodcom_data[product], 0))</f>
         <v>0.97723312392412343</v>
       </c>
@@ -42531,7 +42518,7 @@
         <f t="shared" si="0"/>
         <v>0.91489276799999997</v>
       </c>
-      <c r="H32" s="97">
+      <c r="H32" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B32, prodcom_data[product], 0))</f>
         <v>0.98372184312642852</v>
       </c>
@@ -42616,7 +42603,7 @@
         <f t="shared" si="0"/>
         <v>0.88856497499999998</v>
       </c>
-      <c r="H33" s="97">
+      <c r="H33" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B33, prodcom_data[product], 0))</f>
         <v>0.16881151544376369</v>
       </c>
@@ -42691,7 +42678,7 @@
         <f t="shared" si="0"/>
         <v>0.88675937800000004</v>
       </c>
-      <c r="H34" s="97">
+      <c r="H34" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B34, prodcom_data[product], 0))</f>
         <v>0.9949802605865421</v>
       </c>
@@ -42766,7 +42753,7 @@
         <f t="shared" si="0"/>
         <v>0.88227254300000002</v>
       </c>
-      <c r="H35" s="97">
+      <c r="H35" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B35, prodcom_data[product], 0))</f>
         <v>0.90674928778782138</v>
       </c>
@@ -42855,7 +42842,7 @@
         <f t="shared" si="0"/>
         <v>0.88188415799999997</v>
       </c>
-      <c r="H36" s="97">
+      <c r="H36" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B36, prodcom_data[product], 0))</f>
         <v>0.54958148029233567</v>
       </c>
@@ -42940,7 +42927,7 @@
         <f t="shared" si="0"/>
         <v>0.87233590599999999</v>
       </c>
-      <c r="H37" s="97">
+      <c r="H37" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B37, prodcom_data[product], 0))</f>
         <v>0.50439285712492499</v>
       </c>
@@ -43015,7 +43002,7 @@
         <f t="shared" si="0"/>
         <v>0.84802669900000005</v>
       </c>
-      <c r="H38" s="97">
+      <c r="H38" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B38, prodcom_data[product], 0))</f>
         <v>0.94336652483154892</v>
       </c>
@@ -43100,7 +43087,7 @@
         <f t="shared" si="0"/>
         <v>0.84621718300000004</v>
       </c>
-      <c r="H39" s="97">
+      <c r="H39" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B39, prodcom_data[product], 0))</f>
         <v>0.71535186139088358</v>
       </c>
@@ -43175,7 +43162,7 @@
         <f t="shared" si="0"/>
         <v>0.82143353699999999</v>
       </c>
-      <c r="H40" s="97">
+      <c r="H40" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B40, prodcom_data[product], 0))</f>
         <v>0.97390715616715806</v>
       </c>
@@ -43260,7 +43247,7 @@
         <f t="shared" si="0"/>
         <v>0.79072103000000005</v>
       </c>
-      <c r="H41" s="97">
+      <c r="H41" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B41, prodcom_data[product], 0))</f>
         <v>0.93548794446506622</v>
       </c>
@@ -43345,7 +43332,7 @@
         <f t="shared" si="0"/>
         <v>0.77849552700000002</v>
       </c>
-      <c r="H42" s="97">
+      <c r="H42" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B42, prodcom_data[product], 0))</f>
         <v>0.9345821199560983</v>
       </c>
@@ -43430,7 +43417,7 @@
         <f t="shared" si="0"/>
         <v>0.70506910199999995</v>
       </c>
-      <c r="H43" s="97">
+      <c r="H43" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B43, prodcom_data[product], 0))</f>
         <v>0.85098041922137724</v>
       </c>
@@ -43505,7 +43492,7 @@
         <f t="shared" si="0"/>
         <v>0.683315016</v>
       </c>
-      <c r="H44" s="97">
+      <c r="H44" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B44, prodcom_data[product], 0))</f>
         <v>0.35122892718634474</v>
       </c>
@@ -43580,7 +43567,7 @@
         <f t="shared" si="0"/>
         <v>0.667655569</v>
       </c>
-      <c r="H45" s="97">
+      <c r="H45" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B45, prodcom_data[product], 0))</f>
         <v>0.85514301162071182</v>
       </c>
@@ -43655,7 +43642,7 @@
         <f t="shared" si="0"/>
         <v>0.66734765100000004</v>
       </c>
-      <c r="H46" s="97">
+      <c r="H46" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B46, prodcom_data[product], 0))</f>
         <v>0.80917344833809868</v>
       </c>
@@ -43740,7 +43727,7 @@
         <f t="shared" si="0"/>
         <v>0.64249725999999996</v>
       </c>
-      <c r="H47" s="97">
+      <c r="H47" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B47, prodcom_data[product], 0))</f>
         <v>0.93385612259264728</v>
       </c>
@@ -43824,7 +43811,7 @@
         <f t="shared" si="0"/>
         <v>0.60486187300000005</v>
       </c>
-      <c r="H48" s="97">
+      <c r="H48" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B48, prodcom_data[product], 0))</f>
         <v>0.66130800742337414</v>
       </c>
@@ -43909,7 +43896,7 @@
         <f t="shared" si="0"/>
         <v>0.593659673</v>
       </c>
-      <c r="H49" s="97">
+      <c r="H49" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B49, prodcom_data[product], 0))</f>
         <v>0.84223339185782964</v>
       </c>
@@ -43994,7 +43981,7 @@
         <f t="shared" si="0"/>
         <v>0.507331541</v>
       </c>
-      <c r="H50" s="97">
+      <c r="H50" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B50, prodcom_data[product], 0))</f>
         <v>0.78843905350643284</v>
       </c>
@@ -44069,7 +44056,7 @@
         <f t="shared" si="0"/>
         <v>0.44373955900000001</v>
       </c>
-      <c r="H51" s="97">
+      <c r="H51" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B51, prodcom_data[product], 0))</f>
         <v>0.9014296604554024</v>
       </c>
@@ -44154,7 +44141,7 @@
         <f t="shared" si="0"/>
         <v>0.37760138599999998</v>
       </c>
-      <c r="H52" s="97">
+      <c r="H52" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B52, prodcom_data[product], 0))</f>
         <v>0.11917329138193365</v>
       </c>
@@ -44229,7 +44216,7 @@
         <f t="shared" si="0"/>
         <v>0.334412816</v>
       </c>
-      <c r="H53" s="97">
+      <c r="H53" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B53, prodcom_data[product], 0))</f>
         <v>0.59226283959165005</v>
       </c>
@@ -44296,7 +44283,7 @@
         <f t="shared" si="0"/>
         <v>0.32184670100000001</v>
       </c>
-      <c r="H54" s="97">
+      <c r="H54" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B54, prodcom_data[product], 0))</f>
         <v>0.18642415725740188</v>
       </c>
@@ -44381,7 +44368,7 @@
         <f t="shared" si="0"/>
         <v>0.32163824499999999</v>
       </c>
-      <c r="H55" s="97">
+      <c r="H55" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B55, prodcom_data[product], 0))</f>
         <v>0.27981747008972768</v>
       </c>
@@ -44466,7 +44453,7 @@
         <f t="shared" si="0"/>
         <v>0.31820840700000003</v>
       </c>
-      <c r="H56" s="97">
+      <c r="H56" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B56, prodcom_data[product], 0))</f>
         <v>0.44804616680036363</v>
       </c>
@@ -44551,7 +44538,7 @@
         <f t="shared" si="0"/>
         <v>0.30089410599999999</v>
       </c>
-      <c r="H57" s="97">
+      <c r="H57" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B57, prodcom_data[product], 0))</f>
         <v>0.99702850277831634</v>
       </c>
@@ -44567,7 +44554,7 @@
       <c r="L57" s="79">
         <v>50.49</v>
       </c>
-      <c r="M57" s="98">
+      <c r="M57" s="97">
         <v>1</v>
       </c>
       <c r="N57" s="72">
@@ -44627,7 +44614,7 @@
         <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
-      <c r="H58" s="97">
+      <c r="H58" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B58, prodcom_data[product], 0))</f>
         <v>1</v>
       </c>
@@ -44701,7 +44688,7 @@
         <f t="shared" si="0"/>
         <v>0.25803222599999998</v>
       </c>
-      <c r="H59" s="97">
+      <c r="H59" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B59, prodcom_data[product], 0))</f>
         <v>0.77509698342872879</v>
       </c>
@@ -44785,7 +44772,7 @@
         <f t="shared" si="0"/>
         <v>0.250743096</v>
       </c>
-      <c r="H60" s="97">
+      <c r="H60" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B60, prodcom_data[product], 0))</f>
         <v>0.79762913990660789</v>
       </c>
@@ -44869,7 +44856,7 @@
         <f t="shared" si="0"/>
         <v>0.21527363199999999</v>
       </c>
-      <c r="H61" s="97">
+      <c r="H61" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B61, prodcom_data[product], 0))</f>
         <v>1.1148601794389756E-2</v>
       </c>
@@ -44943,7 +44930,7 @@
         <f t="shared" si="0"/>
         <v>0.24214196815384617</v>
       </c>
-      <c r="H62" s="97">
+      <c r="H62" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B62, prodcom_data[product], 0))</f>
         <v>0.88632047658515611</v>
       </c>
@@ -45028,7 +45015,7 @@
         <f t="shared" si="0"/>
         <v>0.80713989384615381</v>
       </c>
-      <c r="H63" s="97">
+      <c r="H63" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B63, prodcom_data[product], 0))</f>
         <v>0.88632047658515611</v>
       </c>
@@ -45113,7 +45100,7 @@
         <f t="shared" si="0"/>
         <v>1.0891084183783784</v>
       </c>
-      <c r="H64" s="97">
+      <c r="H64" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B64, prodcom_data[product], 0))</f>
         <v>0.87748442629671652</v>
       </c>
@@ -45198,7 +45185,7 @@
         <f t="shared" si="0"/>
         <v>1.2813040216216214</v>
       </c>
-      <c r="H65" s="97">
+      <c r="H65" s="96">
         <f>INDEX(prodcom_data[Local production share of available quantity (PRODQNT + IMPQNT) - EU27 - 2022], MATCH(B65, prodcom_data[product], 0))</f>
         <v>0.87748442629671652</v>
       </c>

</xml_diff>